<commit_message>
data(chf): all refresh 2026-10-01T11:28Z
</commit_message>
<xml_diff>
--- a/logs/chf/raw/efv_outstanding.xlsx
+++ b/logs/chf/raw/efv_outstanding.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Bt-daten\TRES\3 Schuldenmanagement\31 Anleihen\318 Datenbanken und Auswertungen\Web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92248D56-C3A5-4134-AFA9-0E6A0645F6FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4CEBB51-47B6-4B04-8DC8-DF35666386F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ausstehende Anleihen" sheetId="2" r:id="rId1"/>
@@ -294,7 +294,7 @@
     <t>Eidg. 24.06.26/41</t>
   </si>
   <si>
-    <t>Stand per/ Etat au/ stato al/ situation at: 31.08.2026</t>
+    <t>Stand per/ Etat au/ stato al/ situation at: 30.09.2026</t>
   </si>
 </sst>
 </file>
@@ -302,11 +302,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="5">
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="164" formatCode="dd/mm/yy;@"/>
-    <numFmt numFmtId="165" formatCode="0.000%"/>
-    <numFmt numFmtId="166" formatCode="#,##0.000"/>
-    <numFmt numFmtId="167" formatCode="#,##0.0000"/>
+    <numFmt numFmtId="164" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yy;@"/>
+    <numFmt numFmtId="166" formatCode="0.000%"/>
+    <numFmt numFmtId="167" formatCode="#,##0.000"/>
+    <numFmt numFmtId="168" formatCode="#,##0.0000"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -490,12 +490,12 @@
   <cellStyleXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -517,10 +517,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -538,7 +538,7 @@
     <xf numFmtId="3" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -547,16 +547,16 @@
     <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" xfId="7" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="7" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" xfId="7" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="7" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -598,10 +598,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1485,10 +1485,10 @@
         <v>8.7500000000000008E-3</v>
       </c>
       <c r="E26" s="12">
-        <v>715.17000000000007</v>
+        <v>876.41000000000008</v>
       </c>
       <c r="F26" s="12">
-        <v>415.17</v>
+        <v>576.41000000000008</v>
       </c>
       <c r="G26" s="12">
         <v>0</v>
@@ -1674,10 +1674,10 @@
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="E33" s="12">
-        <v>2800.19</v>
+        <v>3007.58</v>
       </c>
       <c r="F33" s="12">
-        <v>2555.19</v>
+        <v>2762.58</v>
       </c>
       <c r="G33" s="12">
         <v>55</v>
@@ -1721,11 +1721,11 @@
       <c r="D35" s="9"/>
       <c r="E35" s="13">
         <f>SUM(E12:E34)</f>
-        <v>80532.639999999999</v>
+        <v>80901.27</v>
       </c>
       <c r="F35" s="13">
         <f>SUM(F12:F34)</f>
-        <v>73655.649999999994</v>
+        <v>74024.28</v>
       </c>
       <c r="G35" s="13">
         <f>SUM(G12:G34)</f>

</xml_diff>